<commit_message>
Schedule and link fixes
</commit_message>
<xml_diff>
--- a/data/Schedule2526.xlsx
+++ b/data/Schedule2526.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cverhoosel/Documents/2_Education/4CBLA30_Energy_Storage_and_Transport/Energy-Storage-and-Transport.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12C8089-BEF9-4A4D-A3FB-8C8E87E9D041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43121BB0-15A5-0C4C-AED4-C286B26AC2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15920" xr2:uid="{2D163C62-21D0-CD47-A46E-4E9962794ACA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="185">
   <si>
     <t>Rooms</t>
   </si>
@@ -246,42 +246,12 @@
     <t>Tutor opening 2</t>
   </si>
   <si>
-    <t>Tutor opening 3</t>
-  </si>
-  <si>
-    <t>Tutor opening 4</t>
-  </si>
-  <si>
     <t>Tutor opening 5</t>
   </si>
   <si>
     <t>Tutor opening 6</t>
   </si>
   <si>
-    <t>Tutor opening 7</t>
-  </si>
-  <si>
-    <t>Tutor opening 8</t>
-  </si>
-  <si>
-    <t>10:30-11:15</t>
-  </si>
-  <si>
-    <t>11:15-12:00</t>
-  </si>
-  <si>
-    <t>12:00-12:45</t>
-  </si>
-  <si>
-    <t>15:15-16:00</t>
-  </si>
-  <si>
-    <t>16:00-16:45</t>
-  </si>
-  <si>
-    <t>16:45-17:30</t>
-  </si>
-  <si>
     <t>II</t>
   </si>
   <si>
@@ -591,9 +561,6 @@
     <t>Gem. N 1.610</t>
   </si>
   <si>
-    <t>Theory sessions, 1 hour or 45 minutes?</t>
-  </si>
-  <si>
     <t>Gemini-Noord 1.710</t>
   </si>
   <si>
@@ -615,15 +582,9 @@
     <t>TR 2.31, TR 2.46, TR 2.48, TR 2.28</t>
   </si>
   <si>
-    <t>Tutor opening, hour or 45 min?</t>
-  </si>
-  <si>
     <t>4,5,7,8</t>
   </si>
   <si>
-    <t>2,9</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
@@ -631,6 +592,9 @@
   </si>
   <si>
     <t>Atlas 5.201, Atlas 7.201, Neuron 0.116, Neuron 0.356</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
 </sst>
 </file>
@@ -1272,7 +1236,7 @@
         <v>39</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -1302,13 +1266,13 @@
         <v>1</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I2" s="26" t="s">
         <v>46</v>
       </c>
       <c r="J2" s="26" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -1326,13 +1290,13 @@
         <v>1</v>
       </c>
       <c r="H3" s="26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I3" s="26" t="s">
         <v>54</v>
       </c>
       <c r="J3" s="26" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1356,7 +1320,7 @@
         <v>64</v>
       </c>
       <c r="J4" s="26" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -1380,7 +1344,7 @@
         <v>63</v>
       </c>
       <c r="J5" s="26" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1397,21 +1361,21 @@
       <c r="E6" s="28"/>
       <c r="F6" s="28"/>
       <c r="G6" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H6" s="26" t="s">
         <v>42</v>
       </c>
       <c r="I6" s="26" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="26" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B7" s="27" t="s">
         <v>6</v>
@@ -1423,16 +1387,16 @@
       <c r="E7" s="28"/>
       <c r="F7" s="28"/>
       <c r="G7" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H7" s="26" t="s">
         <v>42</v>
       </c>
       <c r="I7" s="26" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1443,48 +1407,48 @@
         <v>6</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="28"/>
       <c r="F8" s="28"/>
       <c r="G8" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H8" s="26" t="s">
         <v>42</v>
       </c>
       <c r="I8" s="26" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B9" s="27" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D9" s="28"/>
       <c r="E9" s="28"/>
       <c r="F9" s="28"/>
       <c r="G9" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H9" s="26" t="s">
         <v>42</v>
       </c>
       <c r="I9" s="26" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -1501,21 +1465,21 @@
       <c r="E10" s="28"/>
       <c r="F10" s="28"/>
       <c r="G10" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H10" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I10" s="26" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="J10" s="26" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="26" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>7</v>
@@ -1527,16 +1491,16 @@
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
       <c r="G11" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H11" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I11" s="26" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="J11" s="26" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1547,53 +1511,53 @@
         <v>7</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="28"/>
       <c r="F12" s="28"/>
       <c r="G12" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H12" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I12" s="26" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="J12" s="26" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="26" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B13" s="27" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
       <c r="G13" s="29" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H13" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I13" s="26" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="J13" s="26" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="26" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
@@ -1601,21 +1565,21 @@
       <c r="E14" s="28"/>
       <c r="F14" s="28"/>
       <c r="G14" s="29" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="H14" s="26" t="s">
         <v>43</v>
       </c>
       <c r="I14" s="26" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="J14" s="26" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="26" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -1629,15 +1593,15 @@
         <v>42</v>
       </c>
       <c r="I15" s="26" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="J15" s="26" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="26" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
@@ -1648,18 +1612,18 @@
         <v>4</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I16" s="26" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="J16" s="26" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="26" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="27"/>
@@ -1670,18 +1634,18 @@
         <v>4</v>
       </c>
       <c r="H17" s="26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I17" s="26" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="J17" s="26" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>6</v>
@@ -1700,18 +1664,18 @@
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I18" t="s">
         <v>66</v>
       </c>
       <c r="J18" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>6</v>
@@ -1730,24 +1694,24 @@
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I19" t="s">
         <v>66</v>
       </c>
       <c r="J19" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D20" s="4">
         <v>1</v>
@@ -1760,24 +1724,24 @@
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I20" t="s">
         <v>66</v>
       </c>
       <c r="J20" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D21" s="4">
         <v>2</v>
@@ -1790,18 +1754,18 @@
         <v>1</v>
       </c>
       <c r="H21" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I21" t="s">
         <v>66</v>
       </c>
       <c r="J21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>6</v>
@@ -1820,18 +1784,18 @@
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I22" t="s">
         <v>67</v>
       </c>
       <c r="J22" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>6</v>
@@ -1850,24 +1814,24 @@
         <v>1</v>
       </c>
       <c r="H23" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I23" t="s">
         <v>67</v>
       </c>
       <c r="J23" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D24" s="4">
         <v>1</v>
@@ -1880,24 +1844,24 @@
         <v>1</v>
       </c>
       <c r="H24" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I24" t="s">
         <v>67</v>
       </c>
       <c r="J24" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D25" s="4">
         <v>2</v>
@@ -1910,18 +1874,18 @@
         <v>1</v>
       </c>
       <c r="H25" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I25" t="s">
         <v>67</v>
       </c>
       <c r="J25" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>7</v>
@@ -1940,18 +1904,18 @@
         <v>1</v>
       </c>
       <c r="H26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J26" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>7</v>
@@ -1970,24 +1934,24 @@
         <v>1</v>
       </c>
       <c r="H27" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I27" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J27" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -2000,24 +1964,24 @@
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I28" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J28" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D29" s="4">
         <v>2</v>
@@ -2030,18 +1994,18 @@
         <v>1</v>
       </c>
       <c r="H29" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I29" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J29" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>7</v>
@@ -2060,18 +2024,18 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I30" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J30" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>7</v>
@@ -2090,24 +2054,24 @@
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J31" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -2120,24 +2084,24 @@
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J32" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D33" s="4">
         <v>2</v>
@@ -2150,18 +2114,18 @@
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="I33" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J33" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>6</v>
@@ -2177,21 +2141,21 @@
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H34" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I34" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="J34" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>6</v>
@@ -2207,21 +2171,21 @@
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H35" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I35" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="J35" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>6</v>
@@ -2237,21 +2201,21 @@
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H36" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I36" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J36" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>6</v>
@@ -2267,27 +2231,27 @@
       </c>
       <c r="F37" s="5"/>
       <c r="G37" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H37" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I37" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="J37" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D38" s="4">
         <v>1</v>
@@ -2297,27 +2261,27 @@
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H38" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I38" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="J38" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D39" s="4">
         <v>2</v>
@@ -2327,27 +2291,27 @@
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H39" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I39" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="J39" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D40" s="4">
         <v>1</v>
@@ -2357,27 +2321,27 @@
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H40" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I40" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J40" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D41" s="4">
         <v>2</v>
@@ -2387,21 +2351,21 @@
       </c>
       <c r="F41" s="5"/>
       <c r="G41" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H41" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I41" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="J41" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>6</v>
@@ -2417,21 +2381,21 @@
       </c>
       <c r="F42" s="5"/>
       <c r="G42" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H42" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I42" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="J42" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>6</v>
@@ -2447,21 +2411,21 @@
       </c>
       <c r="F43" s="5"/>
       <c r="G43" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H43" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I43" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="J43" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>6</v>
@@ -2477,21 +2441,21 @@
       </c>
       <c r="F44" s="5"/>
       <c r="G44" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H44" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I44" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="J44" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>6</v>
@@ -2507,27 +2471,27 @@
       </c>
       <c r="F45" s="5"/>
       <c r="G45" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H45" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I45" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="J45" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D46" s="4">
         <v>1</v>
@@ -2537,27 +2501,27 @@
       </c>
       <c r="F46" s="5"/>
       <c r="G46" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H46" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I46" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="J46" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D47" s="4">
         <v>2</v>
@@ -2567,27 +2531,27 @@
       </c>
       <c r="F47" s="5"/>
       <c r="G47" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H47" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I47" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="J47" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D48" s="4">
         <v>1</v>
@@ -2597,27 +2561,27 @@
       </c>
       <c r="F48" s="5"/>
       <c r="G48" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H48" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I48" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J48" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D49" s="4">
         <v>2</v>
@@ -2627,21 +2591,21 @@
       </c>
       <c r="F49" s="5"/>
       <c r="G49" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H49" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I49" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="J49" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>7</v>
@@ -2657,21 +2621,21 @@
       </c>
       <c r="F50" s="5"/>
       <c r="G50" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H50" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I50" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="J50" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>7</v>
@@ -2687,21 +2651,21 @@
       </c>
       <c r="F51" s="5"/>
       <c r="G51" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H51" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I51" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="J51" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>7</v>
@@ -2717,21 +2681,21 @@
       </c>
       <c r="F52" s="5"/>
       <c r="G52" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H52" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I52" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="J52" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>7</v>
@@ -2747,27 +2711,27 @@
       </c>
       <c r="F53" s="5"/>
       <c r="G53" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H53" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I53" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="J53" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D54" s="4">
         <v>1</v>
@@ -2777,27 +2741,27 @@
       </c>
       <c r="F54" s="5"/>
       <c r="G54" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H54" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I54" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="J54" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D55" s="4">
         <v>2</v>
@@ -2807,27 +2771,27 @@
       </c>
       <c r="F55" s="5"/>
       <c r="G55" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H55" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I55" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="J55" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D56" s="4">
         <v>1</v>
@@ -2837,27 +2801,27 @@
       </c>
       <c r="F56" s="5"/>
       <c r="G56" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H56" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I56" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="J56" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D57" s="4">
         <v>2</v>
@@ -2867,21 +2831,21 @@
       </c>
       <c r="F57" s="5"/>
       <c r="G57" s="30" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="H57" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I57" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="J57" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>7</v>
@@ -2897,21 +2861,21 @@
       </c>
       <c r="F58" s="5"/>
       <c r="G58" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H58" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I58" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="J58" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>7</v>
@@ -2927,21 +2891,21 @@
       </c>
       <c r="F59" s="5"/>
       <c r="G59" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H59" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I59" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="J59" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>7</v>
@@ -2957,21 +2921,21 @@
       </c>
       <c r="F60" s="5"/>
       <c r="G60" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H60" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I60" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="J60" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>7</v>
@@ -2987,27 +2951,27 @@
       </c>
       <c r="F61" s="5"/>
       <c r="G61" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H61" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I61" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="J61" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D62" s="4">
         <v>1</v>
@@ -3017,27 +2981,27 @@
       </c>
       <c r="F62" s="5"/>
       <c r="G62" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H62" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I62" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="J62" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D63" s="4">
         <v>2</v>
@@ -3047,27 +3011,27 @@
       </c>
       <c r="F63" s="5"/>
       <c r="G63" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H63" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I63" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J63" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D64" s="4">
         <v>1</v>
@@ -3077,27 +3041,27 @@
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H64" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I64" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="J64" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D65" s="4">
         <v>2</v>
@@ -3107,264 +3071,232 @@
       </c>
       <c r="F65" s="5"/>
       <c r="G65" s="30" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="H65" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I65" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="J65" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B66" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C66" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D66" s="27">
-        <v>1</v>
-      </c>
-      <c r="E66" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="F66" s="28"/>
-      <c r="G66" s="29" t="s">
-        <v>194</v>
+      <c r="C66" s="27"/>
+      <c r="D66" s="28"/>
+      <c r="E66" s="28"/>
+      <c r="F66" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="G66" s="29">
+        <v>9</v>
       </c>
       <c r="H66" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I66" s="26" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="J66" s="26" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B67" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C67" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D67" s="27">
-        <v>2</v>
-      </c>
-      <c r="E67" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="F67" s="28"/>
-      <c r="G67" s="29" t="s">
-        <v>194</v>
+      <c r="C67" s="27"/>
+      <c r="D67" s="28"/>
+      <c r="E67" s="28"/>
+      <c r="F67" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="G67" s="29">
+        <v>9</v>
       </c>
       <c r="H67" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I67" s="26" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="J67" s="26" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B68" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C68" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D68" s="27">
-        <v>1</v>
-      </c>
-      <c r="E68" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="F68" s="28"/>
-      <c r="G68" s="29" t="s">
-        <v>194</v>
+      <c r="C68" s="27"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="G68" s="29">
+        <v>9</v>
       </c>
       <c r="H68" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I68" s="26" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="J68" s="26" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B69" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C69" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D69" s="27">
-        <v>2</v>
-      </c>
-      <c r="E69" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="F69" s="28"/>
-      <c r="G69" s="29" t="s">
-        <v>194</v>
+      <c r="C69" s="27"/>
+      <c r="D69" s="28"/>
+      <c r="E69" s="28"/>
+      <c r="F69" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="G69" s="29">
+        <v>9</v>
       </c>
       <c r="H69" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I69" s="26" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="J69" s="26" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B70" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C70" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D70" s="27">
-        <v>1</v>
-      </c>
-      <c r="E70" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F70" s="28"/>
-      <c r="G70" s="29" t="s">
-        <v>194</v>
+        <v>7</v>
+      </c>
+      <c r="C70" s="27"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="G70" s="29">
+        <v>9</v>
       </c>
       <c r="H70" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I70" s="26" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="J70" s="26" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B71" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C71" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D71" s="27">
-        <v>2</v>
-      </c>
-      <c r="E71" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F71" s="28"/>
-      <c r="G71" s="29" t="s">
-        <v>194</v>
+        <v>7</v>
+      </c>
+      <c r="C71" s="27"/>
+      <c r="D71" s="28"/>
+      <c r="E71" s="28"/>
+      <c r="F71" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="G71" s="29">
+        <v>9</v>
       </c>
       <c r="H71" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I71" s="26" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="J71" s="26" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B72" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C72" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D72" s="27">
-        <v>1</v>
-      </c>
-      <c r="E72" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F72" s="28"/>
-      <c r="G72" s="29" t="s">
-        <v>194</v>
+        <v>7</v>
+      </c>
+      <c r="C72" s="27"/>
+      <c r="D72" s="28"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="G72" s="29">
+        <v>9</v>
       </c>
       <c r="H72" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I72" s="26" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="J72" s="26" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="26" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B73" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C73" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D73" s="27">
-        <v>2</v>
-      </c>
-      <c r="E73" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F73" s="28"/>
-      <c r="G73" s="29" t="s">
-        <v>194</v>
+        <v>7</v>
+      </c>
+      <c r="C73" s="27"/>
+      <c r="D73" s="28"/>
+      <c r="E73" s="28"/>
+      <c r="F73" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="G73" s="29">
+        <v>9</v>
       </c>
       <c r="H73" s="26" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="I73" s="26" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="J73" s="26" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B74" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C74" s="27" t="s">
         <v>44</v>
@@ -3377,24 +3309,24 @@
       </c>
       <c r="F74" s="28"/>
       <c r="G74" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H74" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I74" s="26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J74" s="26" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B75" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C75" s="27" t="s">
         <v>44</v>
@@ -3407,27 +3339,27 @@
       </c>
       <c r="F75" s="28"/>
       <c r="G75" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H75" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I75" s="26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J75" s="26" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B76" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C76" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D76" s="27">
         <v>1</v>
@@ -3437,27 +3369,27 @@
       </c>
       <c r="F76" s="28"/>
       <c r="G76" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H76" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I76" s="26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J76" s="26" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B77" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C77" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D77" s="27">
         <v>2</v>
@@ -3467,24 +3399,24 @@
       </c>
       <c r="F77" s="28"/>
       <c r="G77" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H77" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I77" s="26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J77" s="26" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B78" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C78" s="27" t="s">
         <v>44</v>
@@ -3497,24 +3429,24 @@
       </c>
       <c r="F78" s="28"/>
       <c r="G78" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H78" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I78" s="26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J78" s="26" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B79" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C79" s="27" t="s">
         <v>44</v>
@@ -3527,27 +3459,27 @@
       </c>
       <c r="F79" s="28"/>
       <c r="G79" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H79" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I79" s="26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J79" s="26" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B80" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C80" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D80" s="27">
         <v>1</v>
@@ -3557,27 +3489,27 @@
       </c>
       <c r="F80" s="28"/>
       <c r="G80" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H80" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I80" s="26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J80" s="26" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="26" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B81" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C81" s="27" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D81" s="27">
         <v>2</v>
@@ -3587,224 +3519,256 @@
       </c>
       <c r="F81" s="28"/>
       <c r="G81" s="29" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="H81" s="26" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="I81" s="26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J81" s="26" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B82" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C82" s="27"/>
-      <c r="D82" s="28"/>
-      <c r="E82" s="28"/>
-      <c r="F82" s="28" t="s">
-        <v>169</v>
-      </c>
-      <c r="G82" s="29">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C82" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" s="27">
+        <v>1</v>
+      </c>
+      <c r="E82" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F82" s="28"/>
+      <c r="G82" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H82" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I82" s="26" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="J82" s="26" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B83" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C83" s="27"/>
-      <c r="D83" s="28"/>
-      <c r="E83" s="28"/>
-      <c r="F83" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="G83" s="29">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C83" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83" s="27">
+        <v>2</v>
+      </c>
+      <c r="E83" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F83" s="28"/>
+      <c r="G83" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H83" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B84" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C84" s="27"/>
-      <c r="D84" s="28"/>
-      <c r="E84" s="28"/>
-      <c r="F84" s="28" t="s">
-        <v>171</v>
-      </c>
-      <c r="G84" s="29">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C84" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D84" s="27">
+        <v>1</v>
+      </c>
+      <c r="E84" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F84" s="28"/>
+      <c r="G84" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H84" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B85" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C85" s="27"/>
-      <c r="D85" s="28"/>
-      <c r="E85" s="28"/>
-      <c r="F85" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="G85" s="29">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C85" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D85" s="27">
+        <v>2</v>
+      </c>
+      <c r="E85" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F85" s="28"/>
+      <c r="G85" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H85" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I85" s="26" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="J85" s="26" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B86" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C86" s="27"/>
-      <c r="D86" s="28"/>
-      <c r="E86" s="28"/>
-      <c r="F86" s="28" t="s">
-        <v>169</v>
-      </c>
-      <c r="G86" s="29">
-        <v>9</v>
+      <c r="C86" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D86" s="27">
+        <v>1</v>
+      </c>
+      <c r="E86" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F86" s="28"/>
+      <c r="G86" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H86" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I86" s="26" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="J86" s="26" t="s">
-        <v>196</v>
+        <v>176</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B87" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C87" s="27"/>
-      <c r="D87" s="28"/>
-      <c r="E87" s="28"/>
-      <c r="F87" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="G87" s="29">
-        <v>9</v>
+      <c r="C87" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87" s="27">
+        <v>2</v>
+      </c>
+      <c r="E87" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F87" s="28"/>
+      <c r="G87" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H87" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I87" s="26" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="J87" s="26" t="s">
-        <v>196</v>
+        <v>177</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B88" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C88" s="27"/>
-      <c r="D88" s="28"/>
-      <c r="E88" s="28"/>
-      <c r="F88" s="28" t="s">
-        <v>171</v>
-      </c>
-      <c r="G88" s="29">
-        <v>9</v>
+      <c r="C88" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D88" s="27">
+        <v>1</v>
+      </c>
+      <c r="E88" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F88" s="28"/>
+      <c r="G88" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H88" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I88" s="26" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="J88" s="26" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="26" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B89" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C89" s="27"/>
-      <c r="D89" s="28"/>
-      <c r="E89" s="28"/>
-      <c r="F89" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="G89" s="29">
-        <v>9</v>
+      <c r="C89" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D89" s="27">
+        <v>2</v>
+      </c>
+      <c r="E89" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F89" s="28"/>
+      <c r="G89" s="29" t="s">
+        <v>181</v>
       </c>
       <c r="H89" s="26" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="I89" s="26" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J89" s="26" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
@@ -3920,29 +3884,29 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D5 D18:D81" xr:uid="{1B91A297-B32E-B74E-96DE-8737393A0A8B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D5 D50:D89 D18:D49" xr:uid="{1B91A297-B32E-B74E-96DE-8737393A0A8B}">
       <formula1>"1,2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E110" xr:uid="{DAD12E26-CD57-9C41-AFDC-CF3CC63BFECF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E90:E110 E2:E89" xr:uid="{DAD12E26-CD57-9C41-AFDC-CF3CC63BFECF}">
       <formula1>"odd,even"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H89" xr:uid="{D3DE31F9-3CE9-934A-A952-907E2B684925}">
       <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{9F122CED-5A19-334F-A1E1-49CEF5A955D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B90:B1048576 B2:B89" xr:uid="{9F122CED-5A19-334F-A1E1-49CEF5A955D4}">
       <formula1>"A,B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{F7ED642D-EE31-8841-9AB9-039AD26D8E57}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C90:C1048576 C2:C89" xr:uid="{F7ED642D-EE31-8841-9AB9-039AD26D8E57}">
       <formula1>"I,II"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{54AFF6DA-7454-A045-9947-97FB7EB7B41C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F90:F1048576 F2:F89" xr:uid="{54AFF6DA-7454-A045-9947-97FB7EB7B41C}">
       <formula1>"presentation 1,presentation 2,presentation 3,presentation 4"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="G47:G49 G42:G46 G58:G81" numberStoredAsText="1"/>
+    <ignoredError sqref="G74:G89 G34:G41 G50:G57" numberStoredAsText="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -3954,19 +3918,19 @@
           <x14:formula1>
             <xm:f>Groups!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>E111:E197 D6:D17 D82:D197</xm:sqref>
+          <xm:sqref>E111:E197 D6:D17 D66:D73 D90:D197</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BFDB9108-2B79-FF4B-B3CE-00BF9BD7F2C4}">
+          <x14:formula1>
+            <xm:f>Activities!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A49 A90:A1048576 A58:A89</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FC18148D-06E4-0B45-87D4-23BDA5787143}">
           <x14:formula1>
             <xm:f>Slots!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>I2:I89</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BFDB9108-2B79-FF4B-B3CE-00BF9BD7F2C4}">
-          <x14:formula1>
-            <xm:f>Activities!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A1048576</xm:sqref>
+          <xm:sqref>I2:I49 I58:I89</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3980,14 +3944,10 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
-        <v>183</v>
-      </c>
+      <c r="A1" s="16"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
-        <v>191</v>
-      </c>
+      <c r="A2" s="16"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="16"/>
@@ -4024,7 +3984,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -4034,22 +3994,22 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -4060,7 +4020,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44EEBB0-7826-4541-973F-D32118CA52EC}">
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
@@ -4084,10 +4044,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -4108,18 +4068,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -4140,10 +4100,10 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -4164,23 +4124,23 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
         <v>62</v>
@@ -4188,58 +4148,58 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -4247,7 +4207,7 @@
         <v>63</v>
       </c>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -4255,7 +4215,7 @@
         <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -4263,7 +4223,7 @@
         <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -4271,7 +4231,7 @@
         <v>67</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -4279,7 +4239,7 @@
         <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -4287,135 +4247,103 @@
         <v>69</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" t="s">
         <v>71</v>
-      </c>
-      <c r="B30" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B33" t="s">
-        <v>83</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="B34" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>111</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B40" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>123</v>
-      </c>
-      <c r="B41" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>124</v>
-      </c>
-      <c r="B42" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>125</v>
-      </c>
-      <c r="B43" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>126</v>
-      </c>
-      <c r="B44" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -4458,7 +4386,7 @@
         <v>21</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4472,7 +4400,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4486,7 +4414,7 @@
         <v>21</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4500,7 +4428,7 @@
         <v>20</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4514,7 +4442,7 @@
         <v>21</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4528,7 +4456,7 @@
         <v>20</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4542,7 +4470,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4556,7 +4484,7 @@
         <v>20</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4572,7 +4500,7 @@
         <v>23</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4586,7 +4514,7 @@
         <v>22</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4600,7 +4528,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4614,7 +4542,7 @@
         <v>22</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4628,7 +4556,7 @@
         <v>23</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4642,7 +4570,7 @@
         <v>22</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4656,7 +4584,7 @@
         <v>23</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4670,7 +4598,7 @@
         <v>22</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4688,7 +4616,7 @@
         <v>25</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4702,7 +4630,7 @@
         <v>24</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4716,7 +4644,7 @@
         <v>25</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4730,7 +4658,7 @@
         <v>24</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4744,7 +4672,7 @@
         <v>25</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4758,7 +4686,7 @@
         <v>24</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4772,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4786,7 +4714,7 @@
         <v>24</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4802,7 +4730,7 @@
         <v>27</v>
       </c>
       <c r="F25" s="20" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4816,7 +4744,7 @@
         <v>26</v>
       </c>
       <c r="F26" s="20" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4830,7 +4758,7 @@
         <v>27</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4844,7 +4772,7 @@
         <v>26</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4858,7 +4786,7 @@
         <v>27</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4872,7 +4800,7 @@
         <v>26</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4886,7 +4814,7 @@
         <v>27</v>
       </c>
       <c r="F31" s="21" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -4900,7 +4828,7 @@
         <v>26</v>
       </c>
       <c r="F32" s="21" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -4920,7 +4848,7 @@
         <v>29</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -4934,7 +4862,7 @@
         <v>28</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -4948,7 +4876,7 @@
         <v>29</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -4962,7 +4890,7 @@
         <v>28</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -4976,7 +4904,7 @@
         <v>29</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -4990,7 +4918,7 @@
         <v>28</v>
       </c>
       <c r="F38" s="22" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -5004,7 +4932,7 @@
         <v>29</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -5018,7 +4946,7 @@
         <v>28</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -5034,7 +4962,7 @@
         <v>31</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -5048,7 +4976,7 @@
         <v>30</v>
       </c>
       <c r="F42" s="22" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -5062,7 +4990,7 @@
         <v>31</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -5076,7 +5004,7 @@
         <v>30</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -5090,7 +5018,7 @@
         <v>31</v>
       </c>
       <c r="F45" s="22" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -5104,7 +5032,7 @@
         <v>30</v>
       </c>
       <c r="F46" s="22" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -5118,7 +5046,7 @@
         <v>31</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -5132,7 +5060,7 @@
         <v>30</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -5150,7 +5078,7 @@
         <v>33</v>
       </c>
       <c r="F49" s="24" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -5164,7 +5092,7 @@
         <v>32</v>
       </c>
       <c r="F50" s="24" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -5178,7 +5106,7 @@
         <v>33</v>
       </c>
       <c r="F51" s="25" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -5192,7 +5120,7 @@
         <v>32</v>
       </c>
       <c r="F52" s="25" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -5206,7 +5134,7 @@
         <v>33</v>
       </c>
       <c r="F53" s="24" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -5220,7 +5148,7 @@
         <v>32</v>
       </c>
       <c r="F54" s="24" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -5234,7 +5162,7 @@
         <v>33</v>
       </c>
       <c r="F55" s="25" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -5248,7 +5176,7 @@
         <v>32</v>
       </c>
       <c r="F56" s="25" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
@@ -5264,7 +5192,7 @@
         <v>35</v>
       </c>
       <c r="F57" s="24" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -5278,7 +5206,7 @@
         <v>34</v>
       </c>
       <c r="F58" s="24" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
@@ -5292,7 +5220,7 @@
         <v>35</v>
       </c>
       <c r="F59" s="25" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
@@ -5306,7 +5234,7 @@
         <v>34</v>
       </c>
       <c r="F60" s="25" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -5320,7 +5248,7 @@
         <v>35</v>
       </c>
       <c r="F61" s="24" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -5334,7 +5262,7 @@
         <v>34</v>
       </c>
       <c r="F62" s="24" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -5348,7 +5276,7 @@
         <v>35</v>
       </c>
       <c r="F63" s="25" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -5362,7 +5290,7 @@
         <v>34</v>
       </c>
       <c r="F64" s="25" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>